<commit_message>
fix: third-round audit — F10 conversation ownership enforcement
- F10 (horizontal privilege escalation): GET/DELETE
  /api/conversations/{cid} previously served any caller who knew the
  12-hex conversation id. Now the API verifies the conversation owner
  against X-User-Token; not-owner and not-found both return 404 (no
  existence leak). Frontend history replay now sends the user token.
- Hygiene: ingestion._load_seed made public as load_seed (API layer no
  longer touches a private function).
- Tests: +1 (test_conversation_isolation) -> 14/14 pass.

Docs synced: IMPROVEMENTS (F10 section), traceability (F10 row),
README (security line + 2026-10-27 section); course deliverables
rebuilt (13 test cases incl. TC-013, report totals, summary counts);
SRS/SDD docs updated (security/counts) with PDF re-export; new
validation artifact artifacts/validation_2026-10-27.txt and
docs/交付物清单.md deliverables index.
</commit_message>
<xml_diff>
--- a/docs/课程交付物/系统测试用例.xlsx
+++ b/docs/课程交付物/系统测试用例.xlsx
@@ -2779,81 +2779,133 @@
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
+          <t>CM-testcase-013</t>
+        </is>
+      </c>
+      <c r="B16" s="47" t="inlineStr">
+        <is>
+          <t>会话安全</t>
+        </is>
+      </c>
+      <c r="C16" s="47" t="inlineStr">
+        <is>
+          <t>安全测试</t>
+        </is>
+      </c>
+      <c r="D16" s="47" t="inlineStr">
+        <is>
+          <t>会话读取/删除校验属主,越权返回 404</t>
+        </is>
+      </c>
+      <c r="E16" s="39" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="F16" s="47" t="inlineStr">
+        <is>
+          <t>用户 A 已创建会话</t>
+        </is>
+      </c>
+      <c r="G16" s="46" t="inlineStr">
+        <is>
+          <t>用户 B 携带他人会话 id 访问</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>1.A 提问建立会话 2.B 读取/删除该会话 3.A 读取/删除</t>
+        </is>
+      </c>
+      <c r="I16" s="47" t="inlineStr">
+        <is>
+          <t>B 的读/删均 404(与不存在一致);A 操作 200</t>
+        </is>
+      </c>
+      <c r="J16" s="7" t="inlineStr">
+        <is>
+          <t>同预期</t>
+        </is>
+      </c>
+      <c r="K16" s="7" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L16" s="7" t="inlineStr">
+        <is>
+          <t>Null(无缺陷)</t>
+        </is>
+      </c>
+      <c r="M16" s="34" t="inlineStr">
+        <is>
+          <t>三轮 F10</t>
+        </is>
+      </c>
+      <c r="N16" s="7" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
           <t>CM-testcase-012</t>
         </is>
       </c>
-      <c r="B16" s="47" t="inlineStr">
+      <c r="B17" s="47" t="inlineStr">
         <is>
           <t>回归测试</t>
         </is>
       </c>
-      <c r="C16" s="47" t="inlineStr">
+      <c r="C17" s="47" t="inlineStr">
         <is>
           <t>功能测试</t>
         </is>
       </c>
-      <c r="D16" s="47" t="inlineStr">
+      <c r="D17" s="47" t="inlineStr">
         <is>
           <t>单元测试套件全绿</t>
         </is>
       </c>
-      <c r="E16" s="39" t="inlineStr">
+      <c r="E17" s="39" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="F16" s="47" t="inlineStr">
+      <c r="F17" s="47" t="inlineStr">
         <is>
           <t>开发环境就绪</t>
         </is>
       </c>
-      <c r="G16" s="46" t="inlineStr">
+      <c r="G17" s="7" t="inlineStr">
         <is>
           <t>pytest 全量</t>
         </is>
       </c>
-      <c r="H16" s="7" t="inlineStr">
+      <c r="H17" s="7" t="inlineStr">
         <is>
           <t>1.python -m pytest backend/tests -q</t>
         </is>
       </c>
-      <c r="I16" s="47" t="inlineStr">
+      <c r="I17" s="47" t="inlineStr">
         <is>
           <t>13 passed(冒烟 4 + 完善轮 9)</t>
         </is>
       </c>
-      <c r="J16" s="7" t="inlineStr">
+      <c r="J17" s="7" t="inlineStr">
         <is>
           <t>同预期</t>
         </is>
       </c>
-      <c r="K16" s="7" t="inlineStr">
+      <c r="K17" s="7" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L16" s="7" t="inlineStr">
+      <c r="L17" s="7" t="inlineStr">
         <is>
           <t>Null(无缺陷)</t>
         </is>
       </c>
-      <c r="M16" s="34" t="inlineStr"/>
-      <c r="N16" s="7" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="7" t="n"/>
-      <c r="B17" s="47" t="n"/>
-      <c r="C17" s="47" t="n"/>
-      <c r="D17" s="47" t="n"/>
-      <c r="E17" s="39" t="n"/>
-      <c r="F17" s="47" t="n"/>
-      <c r="G17" s="7" t="n"/>
-      <c r="H17" s="7" t="n"/>
-      <c r="I17" s="47" t="n"/>
-      <c r="J17" s="7" t="n"/>
-      <c r="K17" s="7" t="n"/>
-      <c r="L17" s="7" t="n"/>
-      <c r="M17" s="34" t="n"/>
+      <c r="M17" s="34" t="inlineStr"/>
       <c r="N17" s="7" t="n"/>
     </row>
     <row r="18">

</xml_diff>